<commit_message>
feat(phase2): Add PostgresAdapter reference implementation
</commit_message>
<xml_diff>
--- a/engineering/MAP_V2/00_Architecture/Verification/Phase_08/MAP_CLI_Frontend_Capability_Matrix.xlsx
+++ b/engineering/MAP_V2/00_Architecture/Verification/Phase_08/MAP_CLI_Frontend_Capability_Matrix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Capability Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Action Required" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Required" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Capability Matrix'!$A$1:$I$63</definedName>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,8 +40,13 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -84,8 +89,32 @@
         <bgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E65100"/>
+        <bgColor rgb="00E65100"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C62828"/>
+        <bgColor rgb="00C62828"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E1"/>
+        <bgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEBEE"/>
+        <bgColor rgb="00FFEBEE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -99,11 +128,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -126,6 +183,21 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -491,18 +563,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="37" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -551,6 +625,16 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>Evidence ID</t>
+        </is>
+      </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
+          <t>Rule 19 Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -558,6 +642,16 @@
           <t>Dashboard</t>
         </is>
       </c>
+      <c r="B2" s="10" t="n"/>
+      <c r="C2" s="10" t="n"/>
+      <c r="D2" s="10" t="n"/>
+      <c r="E2" s="10" t="n"/>
+      <c r="F2" s="10" t="n"/>
+      <c r="G2" s="10" t="n"/>
+      <c r="H2" s="10" t="n"/>
+      <c r="I2" s="11" t="n"/>
+      <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -603,6 +697,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -648,6 +744,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -693,6 +791,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -738,6 +838,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -783,6 +885,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -828,6 +932,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -873,6 +979,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>DL-009</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>NEEDS FIX — remap from engine.exceptions to engine.migration_control_exceptions</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -918,6 +1034,16 @@
           <t>NEEDS FIX</t>
         </is>
       </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>DL-007</t>
+        </is>
+      </c>
+      <c r="K10" s="12" t="inlineStr">
+        <is>
+          <t>NEEDS FIX — remap from audit.audit_events to engine.migration_control_execution</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -925,6 +1051,16 @@
           <t>Governance</t>
         </is>
       </c>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
+      <c r="H11" s="10" t="n"/>
+      <c r="I11" s="11" t="n"/>
+      <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -970,6 +1106,16 @@
           <t>NEEDS FIX</t>
         </is>
       </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>DL-007</t>
+        </is>
+      </c>
+      <c r="K12" s="12" t="inlineStr">
+        <is>
+          <t>NEEDS FIX — remap from audit.audit_events to engine.migration_control_execution</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1015,6 +1161,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1060,6 +1208,16 @@
           <t>NEEDS FIX</t>
         </is>
       </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>DL-009</t>
+        </is>
+      </c>
+      <c r="K14" s="12" t="inlineStr">
+        <is>
+          <t>NEEDS FIX — remap from engine.exceptions to engine.migration_control_exceptions</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1105,6 +1263,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1112,6 +1272,16 @@
           <t>Execution Control</t>
         </is>
       </c>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
+      <c r="H16" s="10" t="n"/>
+      <c r="I16" s="11" t="n"/>
+      <c r="J16" s="3" t="n"/>
+      <c r="K16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1157,6 +1327,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1202,6 +1374,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J18" s="3" t="n"/>
+      <c r="K18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1247,6 +1421,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J19" s="3" t="n"/>
+      <c r="K19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1292,6 +1468,16 @@
           <t>PARTIAL</t>
         </is>
       </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>DL-005</t>
+        </is>
+      </c>
+      <c r="K20" s="12" t="inlineStr">
+        <is>
+          <t>PARTIAL — uses engine.batch_execution_checkpoint (batch_id + last_completed_control only)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1337,6 +1523,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J21" s="3" t="n"/>
+      <c r="K21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1344,6 +1532,16 @@
           <t>Execution History</t>
         </is>
       </c>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="10" t="n"/>
+      <c r="H22" s="10" t="n"/>
+      <c r="I22" s="11" t="n"/>
+      <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1389,6 +1587,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1434,6 +1634,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J24" s="3" t="n"/>
+      <c r="K24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1479,6 +1681,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1524,6 +1728,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1569,6 +1775,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1614,6 +1822,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1621,6 +1831,16 @@
           <t>Rule Execution</t>
         </is>
       </c>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="10" t="n"/>
+      <c r="D29" s="10" t="n"/>
+      <c r="E29" s="10" t="n"/>
+      <c r="F29" s="10" t="n"/>
+      <c r="G29" s="10" t="n"/>
+      <c r="H29" s="10" t="n"/>
+      <c r="I29" s="11" t="n"/>
+      <c r="J29" s="3" t="n"/>
+      <c r="K29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -1666,6 +1886,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1711,6 +1933,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J31" s="3" t="n"/>
+      <c r="K31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -1756,6 +1980,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J32" s="3" t="n"/>
+      <c r="K32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1801,6 +2027,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J33" s="3" t="n"/>
+      <c r="K33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1808,6 +2036,16 @@
           <t>Validation Report</t>
         </is>
       </c>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="10" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="10" t="n"/>
+      <c r="G34" s="10" t="n"/>
+      <c r="H34" s="10" t="n"/>
+      <c r="I34" s="11" t="n"/>
+      <c r="J34" s="3" t="n"/>
+      <c r="K34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1853,6 +2091,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -1898,6 +2138,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J36" s="3" t="n"/>
+      <c r="K36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -1943,6 +2185,16 @@
           <t>INVESTIGATE</t>
         </is>
       </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>DL-001</t>
+        </is>
+      </c>
+      <c r="K37" s="13" t="inlineStr">
+        <is>
+          <t>NEEDS UPDATE — engine.unified_scoresDEPRECATED</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -1988,6 +2240,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J38" s="3" t="n"/>
+      <c r="K38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -2033,6 +2287,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J39" s="3" t="n"/>
+      <c r="K39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -2078,6 +2334,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J40" s="3" t="n"/>
+      <c r="K40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2085,6 +2343,16 @@
           <t>Monitoring</t>
         </is>
       </c>
+      <c r="B41" s="10" t="n"/>
+      <c r="C41" s="10" t="n"/>
+      <c r="D41" s="10" t="n"/>
+      <c r="E41" s="10" t="n"/>
+      <c r="F41" s="10" t="n"/>
+      <c r="G41" s="10" t="n"/>
+      <c r="H41" s="10" t="n"/>
+      <c r="I41" s="11" t="n"/>
+      <c r="J41" s="3" t="n"/>
+      <c r="K41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -2132,6 +2400,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J42" s="3" t="n"/>
+      <c r="K42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2177,6 +2447,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J43" s="3" t="n"/>
+      <c r="K43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -2222,6 +2494,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J44" s="3" t="n"/>
+      <c r="K44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -2267,6 +2541,16 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>DL-009</t>
+        </is>
+      </c>
+      <c r="K45" s="12" t="inlineStr">
+        <is>
+          <t>NEEDS FIX — remap from engine.exceptions to engine.migration_control_exceptions</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -2312,6 +2596,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J46" s="3" t="n"/>
+      <c r="K46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2319,6 +2605,16 @@
           <t>Discovery</t>
         </is>
       </c>
+      <c r="B47" s="10" t="n"/>
+      <c r="C47" s="10" t="n"/>
+      <c r="D47" s="10" t="n"/>
+      <c r="E47" s="10" t="n"/>
+      <c r="F47" s="10" t="n"/>
+      <c r="G47" s="10" t="n"/>
+      <c r="H47" s="10" t="n"/>
+      <c r="I47" s="11" t="n"/>
+      <c r="J47" s="3" t="n"/>
+      <c r="K47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -2364,6 +2660,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J48" s="3" t="n"/>
+      <c r="K48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -2409,6 +2707,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J49" s="3" t="n"/>
+      <c r="K49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -2454,6 +2754,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J50" s="3" t="n"/>
+      <c r="K50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -2499,6 +2801,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J51" s="3" t="n"/>
+      <c r="K51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2506,6 +2810,16 @@
           <t>Platform (Auth, Users, Roles, Tasks, Notifications, Settings, Workflows, Calendar, Approvals)</t>
         </is>
       </c>
+      <c r="B52" s="10" t="n"/>
+      <c r="C52" s="10" t="n"/>
+      <c r="D52" s="10" t="n"/>
+      <c r="E52" s="10" t="n"/>
+      <c r="F52" s="10" t="n"/>
+      <c r="G52" s="10" t="n"/>
+      <c r="H52" s="10" t="n"/>
+      <c r="I52" s="11" t="n"/>
+      <c r="J52" s="3" t="n"/>
+      <c r="K52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -2551,6 +2865,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J53" s="3" t="n"/>
+      <c r="K53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -2596,6 +2912,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J54" s="3" t="n"/>
+      <c r="K54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -2641,6 +2959,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J55" s="3" t="n"/>
+      <c r="K55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -2686,6 +3006,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J56" s="3" t="n"/>
+      <c r="K56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -2731,6 +3053,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J57" s="3" t="n"/>
+      <c r="K57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -2776,6 +3100,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J58" s="3" t="n"/>
+      <c r="K58" s="3" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -2821,6 +3147,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J59" s="3" t="n"/>
+      <c r="K59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -2866,6 +3194,8 @@
           <t>EMPTY</t>
         </is>
       </c>
+      <c r="J60" s="3" t="n"/>
+      <c r="K60" s="3" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -2911,6 +3241,8 @@
           <t>EMPTY</t>
         </is>
       </c>
+      <c r="J61" s="3" t="n"/>
+      <c r="K61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -2956,6 +3288,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J62" s="3" t="n"/>
+      <c r="K62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -3001,6 +3335,8 @@
           <t>VERIFIED</t>
         </is>
       </c>
+      <c r="J63" s="3" t="n"/>
+      <c r="K63" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I63"/>
@@ -3025,17 +3361,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="37" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="2" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3079,6 +3418,16 @@
           <t>Action</t>
         </is>
       </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>Evidence ID</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>Rule 19 Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
@@ -3119,6 +3468,8 @@
           <t>Remap query. Map: action-&gt;execution_status, entity_type-&gt;control_id, entity_id-&gt;rule_id, user_email-&gt;SYSTEM, timestamp-&gt;created_at</t>
         </is>
       </c>
+      <c r="I2" s="14" t="n"/>
+      <c r="J2" s="14" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -3159,6 +3510,8 @@
           <t>Remap query. Map: action-&gt;execution_status, entity_type-&gt;control_id, entity_id-&gt;rule_id, user_email-&gt;SYSTEM, timestamp-&gt;created_at</t>
         </is>
       </c>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -3199,6 +3552,8 @@
           <t>Remap query. Map: status-&gt;gate_result, requested_by-&gt;approved_by, entity_type-&gt;client_name, entity_id-&gt;batch_id</t>
         </is>
       </c>
+      <c r="I4" s="14" t="n"/>
+      <c r="J4" s="14" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -3239,6 +3594,8 @@
           <t>Remap query. Map: reason-&gt;cause, status-&gt;failure_scope, requested_by-&gt;SYSTEM, entity_type-&gt;control_id, entity_id-&gt;rule_id</t>
         </is>
       </c>
+      <c r="I5" s="14" t="n"/>
+      <c r="J5" s="14" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -3279,6 +3636,8 @@
           <t>Option A: Use batch_execution_checkpoint (partial data). Option B: Create lifecycle table</t>
         </is>
       </c>
+      <c r="I6" s="14" t="n"/>
+      <c r="J6" s="14" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -3319,6 +3678,8 @@
           <t>Option A: Trace source, adapt mapping. Option B: BLOCK per RULE 16</t>
         </is>
       </c>
+      <c r="I7" s="14" t="n"/>
+      <c r="J7" s="14" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -3359,6 +3720,8 @@
           <t>Platform feature - no MAP CLI data flows here. Keep as-is.</t>
         </is>
       </c>
+      <c r="I8" s="14" t="n"/>
+      <c r="J8" s="14" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -3399,6 +3762,8 @@
           <t>Platform feature - no MAP CLI data flows here. Keep as-is.</t>
         </is>
       </c>
+      <c r="I9" s="14" t="n"/>
+      <c r="J9" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>